<commit_message>
change name of patreg + new vars desc
</commit_message>
<xml_diff>
--- a/static/files/meta_variables.xlsx
+++ b/static/files/meta_variables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lina\STATISTIK\Projects\20210525_shfdb4\dm\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC082D99-BD3A-4620-AB59-C83B35AC7311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D54350-961B-4BB4-8D8C-8FB325E734A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -763,9 +763,6 @@
     <t>beats/min</t>
   </si>
   <si>
-    <t>Hb</t>
-  </si>
-  <si>
     <t>g/L</t>
   </si>
   <si>
@@ -1096,9 +1093,6 @@
     <t>Valvular disease</t>
   </si>
   <si>
-    <t>Renal failure</t>
-  </si>
-  <si>
     <t>Hyperkalemia</t>
   </si>
   <si>
@@ -1123,12 +1117,6 @@
     <t>Depression</t>
   </si>
   <si>
-    <t>Malignant cancer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muscoloskeletal/connective tissue diseases </t>
-  </si>
-  <si>
     <t>Alcohol abuse</t>
   </si>
   <si>
@@ -1171,9 +1159,6 @@
     <t>Pneumonia hospitalization</t>
   </si>
   <si>
-    <t>Renal Failure hospitalization</t>
-  </si>
-  <si>
     <t>Malignant cancer hospitalization</t>
   </si>
   <si>
@@ -1286,6 +1271,21 @@
   </si>
   <si>
     <t>BMI (imputed)</t>
+  </si>
+  <si>
+    <t>Hemoglobin</t>
+  </si>
+  <si>
+    <t>Kidney disease</t>
+  </si>
+  <si>
+    <t>Kidney disease hospitalization</t>
+  </si>
+  <si>
+    <t>Malignant cancer within 3 years</t>
+  </si>
+  <si>
+    <t>Muscoloskeletal/connective tissue diseases within 3 years</t>
   </si>
 </sst>
 </file>
@@ -1737,7 +1737,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="E8" t="s">
         <v>208</v>
@@ -1779,7 +1779,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C11" t="s">
         <v>210</v>
@@ -1894,7 +1894,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1935,7 +1935,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>211</v>
@@ -2012,10 +2012,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
+        <v>417</v>
+      </c>
+      <c r="C33" t="s">
         <v>247</v>
-      </c>
-      <c r="C33" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -2023,13 +2023,13 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
+        <v>248</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -2037,10 +2037,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
+        <v>251</v>
+      </c>
+      <c r="C35" t="s">
         <v>252</v>
-      </c>
-      <c r="C35" t="s">
-        <v>253</v>
       </c>
       <c r="D35" t="s">
         <v>234</v>
@@ -2051,10 +2051,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
+        <v>253</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="D36" s="3"/>
     </row>
@@ -2063,10 +2063,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
+        <v>255</v>
+      </c>
+      <c r="C37" t="s">
         <v>256</v>
-      </c>
-      <c r="C37" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -2074,10 +2074,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
+        <v>257</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>259</v>
       </c>
       <c r="D38" s="3"/>
     </row>
@@ -2086,10 +2086,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -2097,7 +2097,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C40" t="s">
         <v>210</v>
@@ -2111,10 +2111,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
+        <v>261</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>262</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>263</v>
       </c>
       <c r="D41" t="s">
         <v>211</v>
@@ -2125,13 +2125,13 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
+        <v>263</v>
+      </c>
+      <c r="C42" t="s">
         <v>264</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>265</v>
-      </c>
-      <c r="D42" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -2139,10 +2139,10 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
+        <v>266</v>
+      </c>
+      <c r="D43" t="s">
         <v>267</v>
-      </c>
-      <c r="D43" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -2150,7 +2150,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>211</v>
@@ -2161,7 +2161,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>211</v>
@@ -2172,13 +2172,13 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
+        <v>298</v>
+      </c>
+      <c r="D46" t="s">
+        <v>282</v>
+      </c>
+      <c r="E46" t="s">
         <v>299</v>
-      </c>
-      <c r="D46" t="s">
-        <v>283</v>
-      </c>
-      <c r="E46" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -2186,16 +2186,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
+        <v>300</v>
+      </c>
+      <c r="C47" t="s">
         <v>301</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
+        <v>282</v>
+      </c>
+      <c r="E47" t="s">
         <v>302</v>
-      </c>
-      <c r="D47" t="s">
-        <v>283</v>
-      </c>
-      <c r="E47" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -2203,13 +2203,13 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="D48" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E48" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -2217,7 +2217,7 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -2225,7 +2225,7 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -2233,7 +2233,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D51" t="s">
         <v>234</v>
@@ -2244,7 +2244,7 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -2252,10 +2252,10 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
+        <v>271</v>
+      </c>
+      <c r="C53" t="s">
         <v>272</v>
-      </c>
-      <c r="C53" t="s">
-        <v>273</v>
       </c>
       <c r="D53" t="s">
         <v>234</v>
@@ -2266,7 +2266,7 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D54" t="s">
         <v>234</v>
@@ -2277,7 +2277,7 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -2285,7 +2285,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D56" t="s">
         <v>211</v>
@@ -2296,13 +2296,13 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
+        <v>276</v>
+      </c>
+      <c r="C57" t="s">
+        <v>272</v>
+      </c>
+      <c r="E57" t="s">
         <v>277</v>
-      </c>
-      <c r="C57" t="s">
-        <v>273</v>
-      </c>
-      <c r="E57" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -2310,7 +2310,7 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -2318,7 +2318,7 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -2326,13 +2326,13 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C60" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E60" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -2340,10 +2340,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
+        <v>281</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>283</v>
       </c>
       <c r="E61" s="1"/>
     </row>
@@ -2352,13 +2352,13 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C62" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E62" s="1"/>
     </row>
@@ -2367,7 +2367,7 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -2375,7 +2375,7 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -2383,7 +2383,7 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -2391,13 +2391,13 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C66" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E66" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -2405,7 +2405,7 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -2413,10 +2413,10 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
+        <v>289</v>
+      </c>
+      <c r="D68" s="5" t="s">
         <v>290</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -2424,16 +2424,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C69" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E69" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2441,7 +2441,7 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -2449,7 +2449,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2457,10 +2457,10 @@
         <v>70</v>
       </c>
       <c r="B72" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="E72" t="s">
         <v>295</v>
-      </c>
-      <c r="E72" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -2468,7 +2468,7 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -2476,7 +2476,7 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -2484,10 +2484,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D75" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -2495,10 +2495,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="D76" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2506,13 +2506,13 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="C77" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D77" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -2520,7 +2520,7 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="D78" t="s">
         <v>211</v>
@@ -2531,7 +2531,7 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -2539,13 +2539,13 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
+        <v>305</v>
+      </c>
+      <c r="D80" t="s">
         <v>306</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>307</v>
-      </c>
-      <c r="E80" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -2553,13 +2553,13 @@
         <v>79</v>
       </c>
       <c r="B81" t="s">
+        <v>308</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D81" s="2" t="s">
+      <c r="E81" t="s">
         <v>310</v>
-      </c>
-      <c r="E81" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -2567,13 +2567,13 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D82" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E82" t="s">
         <v>312</v>
-      </c>
-      <c r="E82" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -2581,13 +2581,13 @@
         <v>81</v>
       </c>
       <c r="B83" t="s">
+        <v>313</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E83" t="s">
         <v>314</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="E83" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -2595,13 +2595,13 @@
         <v>82</v>
       </c>
       <c r="B84" t="s">
+        <v>315</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E84" t="s">
         <v>316</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="E84" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -2609,10 +2609,10 @@
         <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2620,10 +2620,10 @@
         <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2631,13 +2631,13 @@
         <v>85</v>
       </c>
       <c r="B87" t="s">
+        <v>319</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E87" t="s">
         <v>320</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="E87" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -2645,13 +2645,13 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
+        <v>321</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E88" t="s">
         <v>322</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="E88" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -2659,13 +2659,13 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E89" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -2673,10 +2673,10 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
+        <v>324</v>
+      </c>
+      <c r="E90" t="s">
         <v>325</v>
-      </c>
-      <c r="E90" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2684,7 +2684,7 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -2692,7 +2692,7 @@
         <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -2700,7 +2700,7 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -2708,13 +2708,13 @@
         <v>92</v>
       </c>
       <c r="B94" t="s">
+        <v>329</v>
+      </c>
+      <c r="C94" t="s">
         <v>330</v>
       </c>
-      <c r="C94" t="s">
+      <c r="E94" t="s">
         <v>331</v>
-      </c>
-      <c r="E94" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2722,13 +2722,13 @@
         <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="C95" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E95" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -2763,7 +2763,7 @@
         <v>97</v>
       </c>
       <c r="B99" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -2779,10 +2779,10 @@
         <v>99</v>
       </c>
       <c r="B101" t="s">
+        <v>248</v>
+      </c>
+      <c r="C101" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -2801,7 +2801,7 @@
         <v>101</v>
       </c>
       <c r="B103" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -2809,21 +2809,21 @@
         <v>102</v>
       </c>
       <c r="B104" t="s">
+        <v>329</v>
+      </c>
+      <c r="C104" t="s">
         <v>330</v>
-      </c>
-      <c r="C104" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="B105" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="C105" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -2831,10 +2831,10 @@
         <v>103</v>
       </c>
       <c r="B106" t="s">
+        <v>255</v>
+      </c>
+      <c r="C106" t="s">
         <v>256</v>
-      </c>
-      <c r="C106" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -2842,7 +2842,7 @@
         <v>104</v>
       </c>
       <c r="B107" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C107" s="3"/>
     </row>
@@ -2851,7 +2851,7 @@
         <v>105</v>
       </c>
       <c r="B108" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -2859,7 +2859,7 @@
         <v>106</v>
       </c>
       <c r="B109" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C109" s="3"/>
     </row>
@@ -2868,7 +2868,7 @@
         <v>107</v>
       </c>
       <c r="B110" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -2876,7 +2876,7 @@
         <v>108</v>
       </c>
       <c r="B111" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -2884,7 +2884,7 @@
         <v>109</v>
       </c>
       <c r="B112" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
@@ -2892,7 +2892,7 @@
         <v>110</v>
       </c>
       <c r="B113" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
@@ -2900,10 +2900,10 @@
         <v>111</v>
       </c>
       <c r="B114" t="s">
+        <v>334</v>
+      </c>
+      <c r="E114" t="s">
         <v>335</v>
-      </c>
-      <c r="E114" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
@@ -2911,7 +2911,7 @@
         <v>112</v>
       </c>
       <c r="B115" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -2919,7 +2919,7 @@
         <v>113</v>
       </c>
       <c r="B116" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
@@ -2927,10 +2927,10 @@
         <v>114</v>
       </c>
       <c r="B117" t="s">
+        <v>338</v>
+      </c>
+      <c r="E117" t="s">
         <v>339</v>
-      </c>
-      <c r="E117" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
@@ -2938,10 +2938,10 @@
         <v>115</v>
       </c>
       <c r="B118" t="s">
+        <v>340</v>
+      </c>
+      <c r="E118" t="s">
         <v>341</v>
-      </c>
-      <c r="E118" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
@@ -2949,10 +2949,10 @@
         <v>116</v>
       </c>
       <c r="B119" t="s">
+        <v>342</v>
+      </c>
+      <c r="C119" t="s">
         <v>343</v>
-      </c>
-      <c r="C119" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
@@ -2960,7 +2960,7 @@
         <v>117</v>
       </c>
       <c r="B120" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
@@ -2974,7 +2974,7 @@
         <v>206</v>
       </c>
       <c r="E121" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
@@ -2982,13 +2982,13 @@
         <v>119</v>
       </c>
       <c r="B122" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C122" t="s">
         <v>206</v>
       </c>
       <c r="E122" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
@@ -2999,7 +2999,7 @@
         <v>224</v>
       </c>
       <c r="E123" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
@@ -3007,10 +3007,10 @@
         <v>121</v>
       </c>
       <c r="B124" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E124" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
@@ -3018,10 +3018,10 @@
         <v>122</v>
       </c>
       <c r="B125" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E125" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
@@ -3029,10 +3029,10 @@
         <v>123</v>
       </c>
       <c r="B126" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E126" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -3040,10 +3040,10 @@
         <v>124</v>
       </c>
       <c r="B127" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E127" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
@@ -3051,10 +3051,10 @@
         <v>125</v>
       </c>
       <c r="B128" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E128" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
@@ -3062,10 +3062,10 @@
         <v>126</v>
       </c>
       <c r="B129" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E129" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
@@ -3073,10 +3073,10 @@
         <v>127</v>
       </c>
       <c r="B130" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E130" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
@@ -3084,10 +3084,10 @@
         <v>128</v>
       </c>
       <c r="B131" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E131" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
@@ -3095,10 +3095,10 @@
         <v>129</v>
       </c>
       <c r="B132" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E132" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
@@ -3106,10 +3106,10 @@
         <v>130</v>
       </c>
       <c r="B133" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E133" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
@@ -3117,10 +3117,10 @@
         <v>131</v>
       </c>
       <c r="B134" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E134" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
@@ -3128,10 +3128,10 @@
         <v>132</v>
       </c>
       <c r="B135" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E135" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
@@ -3139,10 +3139,10 @@
         <v>133</v>
       </c>
       <c r="B136" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E136" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
@@ -3150,10 +3150,10 @@
         <v>134</v>
       </c>
       <c r="B137" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E137" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
@@ -3161,10 +3161,10 @@
         <v>135</v>
       </c>
       <c r="B138" t="s">
-        <v>358</v>
+        <v>418</v>
       </c>
       <c r="E138" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
@@ -3172,10 +3172,10 @@
         <v>136</v>
       </c>
       <c r="B139" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E139" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
@@ -3183,10 +3183,10 @@
         <v>137</v>
       </c>
       <c r="B140" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E140" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
@@ -3194,10 +3194,10 @@
         <v>138</v>
       </c>
       <c r="B141" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E141" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
@@ -3205,10 +3205,10 @@
         <v>139</v>
       </c>
       <c r="B142" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E142" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
@@ -3216,10 +3216,10 @@
         <v>140</v>
       </c>
       <c r="B143" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E143" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
@@ -3227,10 +3227,10 @@
         <v>141</v>
       </c>
       <c r="B144" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E144" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
@@ -3238,10 +3238,10 @@
         <v>142</v>
       </c>
       <c r="B145" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E145" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
@@ -3249,10 +3249,10 @@
         <v>143</v>
       </c>
       <c r="B146" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E146" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
@@ -3260,10 +3260,10 @@
         <v>144</v>
       </c>
       <c r="B147" t="s">
-        <v>367</v>
+        <v>420</v>
       </c>
       <c r="E147" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
@@ -3271,10 +3271,10 @@
         <v>145</v>
       </c>
       <c r="B148" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
       <c r="E148" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
@@ -3282,10 +3282,10 @@
         <v>146</v>
       </c>
       <c r="B149" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E149" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
@@ -3293,10 +3293,10 @@
         <v>147</v>
       </c>
       <c r="B150" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="E150" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
@@ -3304,10 +3304,10 @@
         <v>148</v>
       </c>
       <c r="B151" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="E151" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
@@ -3315,10 +3315,10 @@
         <v>149</v>
       </c>
       <c r="B152" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="E152" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
@@ -3329,7 +3329,7 @@
         <v>206</v>
       </c>
       <c r="E153" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
@@ -3337,10 +3337,10 @@
         <v>151</v>
       </c>
       <c r="B154" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="E154" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
@@ -3348,10 +3348,10 @@
         <v>152</v>
       </c>
       <c r="B155" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="E155" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
@@ -3362,7 +3362,7 @@
         <v>206</v>
       </c>
       <c r="E156" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
@@ -3370,10 +3370,10 @@
         <v>154</v>
       </c>
       <c r="B157" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E157" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
@@ -3384,7 +3384,7 @@
         <v>206</v>
       </c>
       <c r="E158" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
@@ -3392,10 +3392,10 @@
         <v>156</v>
       </c>
       <c r="B159" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="E159" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
@@ -3406,7 +3406,7 @@
         <v>206</v>
       </c>
       <c r="E160" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
@@ -3414,10 +3414,10 @@
         <v>158</v>
       </c>
       <c r="B161" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="E161" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
@@ -3428,7 +3428,7 @@
         <v>206</v>
       </c>
       <c r="E162" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
@@ -3436,10 +3436,10 @@
         <v>160</v>
       </c>
       <c r="B163" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="E163" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
@@ -3450,7 +3450,7 @@
         <v>206</v>
       </c>
       <c r="E164" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
@@ -3458,10 +3458,10 @@
         <v>162</v>
       </c>
       <c r="B165" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E165" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
@@ -3472,7 +3472,7 @@
         <v>206</v>
       </c>
       <c r="E166" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
@@ -3480,10 +3480,10 @@
         <v>164</v>
       </c>
       <c r="B167" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="E167" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
@@ -3494,7 +3494,7 @@
         <v>206</v>
       </c>
       <c r="E168" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
@@ -3505,7 +3505,7 @@
         <v>206</v>
       </c>
       <c r="E169" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
@@ -3513,10 +3513,10 @@
         <v>167</v>
       </c>
       <c r="B170" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="E170" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
@@ -3527,7 +3527,7 @@
         <v>206</v>
       </c>
       <c r="E171" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
@@ -3535,10 +3535,10 @@
         <v>169</v>
       </c>
       <c r="B172" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="E172" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
@@ -3549,7 +3549,7 @@
         <v>206</v>
       </c>
       <c r="E173" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
@@ -3557,10 +3557,10 @@
         <v>171</v>
       </c>
       <c r="B174" t="s">
-        <v>383</v>
+        <v>419</v>
       </c>
       <c r="E174" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
@@ -3571,7 +3571,7 @@
         <v>206</v>
       </c>
       <c r="E175" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
@@ -3579,10 +3579,10 @@
         <v>173</v>
       </c>
       <c r="B176" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="E176" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
@@ -3593,7 +3593,7 @@
         <v>206</v>
       </c>
       <c r="E177" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
@@ -3601,10 +3601,10 @@
         <v>175</v>
       </c>
       <c r="B178" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E178" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
@@ -3615,7 +3615,7 @@
         <v>206</v>
       </c>
       <c r="E179" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
@@ -3623,10 +3623,10 @@
         <v>177</v>
       </c>
       <c r="B180" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E180" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
@@ -3637,7 +3637,7 @@
         <v>206</v>
       </c>
       <c r="E181" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
@@ -3645,10 +3645,10 @@
         <v>179</v>
       </c>
       <c r="B182" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E182" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
@@ -3659,7 +3659,7 @@
         <v>206</v>
       </c>
       <c r="E183" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
@@ -3667,10 +3667,10 @@
         <v>181</v>
       </c>
       <c r="B184" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="E184" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
@@ -3681,7 +3681,7 @@
         <v>206</v>
       </c>
       <c r="E185" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
@@ -3689,10 +3689,10 @@
         <v>183</v>
       </c>
       <c r="B186" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="E186" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
@@ -3703,7 +3703,7 @@
         <v>206</v>
       </c>
       <c r="E187" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
@@ -3711,10 +3711,10 @@
         <v>185</v>
       </c>
       <c r="B188" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="E188" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
@@ -3725,7 +3725,7 @@
         <v>206</v>
       </c>
       <c r="E189" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
@@ -3733,10 +3733,10 @@
         <v>187</v>
       </c>
       <c r="B190" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="E190" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
@@ -3747,7 +3747,7 @@
         <v>206</v>
       </c>
       <c r="E191" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
@@ -3755,10 +3755,10 @@
         <v>189</v>
       </c>
       <c r="B192" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E192" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
@@ -3766,10 +3766,10 @@
         <v>190</v>
       </c>
       <c r="B193" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="E193" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
@@ -3777,10 +3777,10 @@
         <v>191</v>
       </c>
       <c r="B194" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="E194" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.25">
@@ -3788,7 +3788,7 @@
         <v>192</v>
       </c>
       <c r="B195" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.25">
@@ -3796,7 +3796,7 @@
         <v>193</v>
       </c>
       <c r="B196" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.25">
@@ -3804,7 +3804,7 @@
         <v>194</v>
       </c>
       <c r="B197" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>